<commit_message>
add: nb_files property for dataset entity
- add nb_files to dataset schema, type, column, info component and datatable
- add nb_files icon (copy) and color in constants and scss
- add nb_files to evolution columnCleanNames and attributs-def
- fix evolution schema: accept number type in old_value/new_value
- fix evolution: convert variable names from snake_case to camelCase for consistent icon/label display
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9262B4DA-1771-8744-82DE-8494BD335BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225553FA-C012-F041-B23D-9037C1595045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2440" yWindow="500" windowWidth="26360" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="209">
   <si>
     <t>id</t>
   </si>
@@ -644,6 +644,9 @@
   </si>
   <si>
     <t>dataset/accident_route.xlsx</t>
+  </si>
+  <si>
+    <t>nb_files</t>
   </si>
 </sst>
 </file>
@@ -722,9 +725,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:S21" totalsRowShown="0">
-  <autoFilter ref="A1:S21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:T21" totalsRowShown="0">
+  <autoFilter ref="A1:T21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -742,6 +745,7 @@
     <tableColumn id="16" xr3:uid="{ED3587E2-4956-D94E-81CF-A84E6EFAC119}" name="delivery_format"/>
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
+    <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_files"/>
     <tableColumn id="18" xr3:uid="{4730D97E-AE17-A44B-9512-0BF292D5AFB4}" name="tag_ids"/>
     <tableColumn id="19" xr3:uid="{288E2992-818F-AA4B-8F92-E9D2F7E670E8}" name="doc_ids"/>
   </tableColumns>
@@ -1036,7 +1040,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1055,11 +1059,12 @@
     <col min="15" max="15" width="16" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1112,13 +1117,16 @@
         <v>18</v>
       </c>
       <c r="R1" t="s">
+        <v>208</v>
+      </c>
+      <c r="S1" t="s">
         <v>103</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1161,11 +1169,11 @@
       <c r="Q2" t="s">
         <v>182</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1217,11 +1225,11 @@
       <c r="Q3" t="s">
         <v>183</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1263,11 +1271,11 @@
       <c r="Q4" t="s">
         <v>184</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1303,11 +1311,11 @@
       <c r="Q5" t="s">
         <v>185</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1353,14 +1361,14 @@
       <c r="Q6" t="s">
         <v>186</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>144</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1406,14 +1414,14 @@
       <c r="Q7" t="s">
         <v>187</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>145</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1456,11 +1464,11 @@
       <c r="Q8" t="s">
         <v>188</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1506,11 +1514,11 @@
       <c r="Q9" t="s">
         <v>189</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1553,11 +1561,11 @@
       <c r="Q10" t="s">
         <v>190</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1603,11 +1611,11 @@
       <c r="Q11" t="s">
         <v>191</v>
       </c>
-      <c r="R11" t="s">
+      <c r="S11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1650,14 +1658,14 @@
       <c r="O12" t="s">
         <v>38</v>
       </c>
-      <c r="R12" t="s">
+      <c r="S12" t="s">
         <v>149</v>
       </c>
-      <c r="S12" t="s">
+      <c r="T12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1703,11 +1711,11 @@
       <c r="Q13" t="s">
         <v>192</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1753,11 +1761,11 @@
       <c r="Q14" t="s">
         <v>193</v>
       </c>
-      <c r="S14" t="s">
+      <c r="T14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1803,8 +1811,11 @@
       <c r="Q15" t="s">
         <v>194</v>
       </c>
+      <c r="R15">
+        <v>3</v>
+      </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1841,11 +1852,11 @@
       <c r="O16" t="s">
         <v>20</v>
       </c>
-      <c r="R16" t="s">
+      <c r="S16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1891,11 +1902,11 @@
       <c r="Q17" t="s">
         <v>195</v>
       </c>
-      <c r="R17" t="s">
+      <c r="S17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -1941,14 +1952,17 @@
       <c r="Q18" t="s">
         <v>196</v>
       </c>
-      <c r="R18" t="s">
+      <c r="R18">
+        <v>13</v>
+      </c>
+      <c r="S18" t="s">
         <v>153</v>
       </c>
-      <c r="S18" t="s">
+      <c r="T18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1994,14 +2008,14 @@
       <c r="Q19" t="s">
         <v>197</v>
       </c>
-      <c r="R19" t="s">
+      <c r="S19" t="s">
         <v>154</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2047,11 +2061,11 @@
       <c r="Q20" t="s">
         <v>198</v>
       </c>
-      <c r="R20" t="s">
+      <c r="S20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
add: nb_files property for dataset entity (#94)
* add: nb_files property for dataset entity

- add nb_files to dataset schema, type, column, info component and datatable
- add nb_files icon (copy) and color in constants and scss
- add nb_files to evolution columnCleanNames and attributs-def
- fix evolution schema: accept number type in old_value/new_value
- fix evolution: convert variable names from snake_case to camelCase for consistent icon/label display

* delete: remove pull request template file

* refactor: update CI workflow for improved structure and clarity

* change: update Svelte check to include router index update

* change: update Svelte check to generate router index separately
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9262B4DA-1771-8744-82DE-8494BD335BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225553FA-C012-F041-B23D-9037C1595045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2440" yWindow="500" windowWidth="26360" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="209">
   <si>
     <t>id</t>
   </si>
@@ -644,6 +644,9 @@
   </si>
   <si>
     <t>dataset/accident_route.xlsx</t>
+  </si>
+  <si>
+    <t>nb_files</t>
   </si>
 </sst>
 </file>
@@ -722,9 +725,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:S21" totalsRowShown="0">
-  <autoFilter ref="A1:S21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:T21" totalsRowShown="0">
+  <autoFilter ref="A1:T21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -742,6 +745,7 @@
     <tableColumn id="16" xr3:uid="{ED3587E2-4956-D94E-81CF-A84E6EFAC119}" name="delivery_format"/>
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
+    <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_files"/>
     <tableColumn id="18" xr3:uid="{4730D97E-AE17-A44B-9512-0BF292D5AFB4}" name="tag_ids"/>
     <tableColumn id="19" xr3:uid="{288E2992-818F-AA4B-8F92-E9D2F7E670E8}" name="doc_ids"/>
   </tableColumns>
@@ -1036,7 +1040,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1055,11 +1059,12 @@
     <col min="15" max="15" width="16" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1112,13 +1117,16 @@
         <v>18</v>
       </c>
       <c r="R1" t="s">
+        <v>208</v>
+      </c>
+      <c r="S1" t="s">
         <v>103</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1161,11 +1169,11 @@
       <c r="Q2" t="s">
         <v>182</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1217,11 +1225,11 @@
       <c r="Q3" t="s">
         <v>183</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1263,11 +1271,11 @@
       <c r="Q4" t="s">
         <v>184</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1303,11 +1311,11 @@
       <c r="Q5" t="s">
         <v>185</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1353,14 +1361,14 @@
       <c r="Q6" t="s">
         <v>186</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>144</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1406,14 +1414,14 @@
       <c r="Q7" t="s">
         <v>187</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>145</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1456,11 +1464,11 @@
       <c r="Q8" t="s">
         <v>188</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1506,11 +1514,11 @@
       <c r="Q9" t="s">
         <v>189</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1553,11 +1561,11 @@
       <c r="Q10" t="s">
         <v>190</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1603,11 +1611,11 @@
       <c r="Q11" t="s">
         <v>191</v>
       </c>
-      <c r="R11" t="s">
+      <c r="S11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1650,14 +1658,14 @@
       <c r="O12" t="s">
         <v>38</v>
       </c>
-      <c r="R12" t="s">
+      <c r="S12" t="s">
         <v>149</v>
       </c>
-      <c r="S12" t="s">
+      <c r="T12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1703,11 +1711,11 @@
       <c r="Q13" t="s">
         <v>192</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1753,11 +1761,11 @@
       <c r="Q14" t="s">
         <v>193</v>
       </c>
-      <c r="S14" t="s">
+      <c r="T14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1803,8 +1811,11 @@
       <c r="Q15" t="s">
         <v>194</v>
       </c>
+      <c r="R15">
+        <v>3</v>
+      </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1841,11 +1852,11 @@
       <c r="O16" t="s">
         <v>20</v>
       </c>
-      <c r="R16" t="s">
+      <c r="S16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1891,11 +1902,11 @@
       <c r="Q17" t="s">
         <v>195</v>
       </c>
-      <c r="R17" t="s">
+      <c r="S17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -1941,14 +1952,17 @@
       <c r="Q18" t="s">
         <v>196</v>
       </c>
-      <c r="R18" t="s">
+      <c r="R18">
+        <v>13</v>
+      </c>
+      <c r="S18" t="s">
         <v>153</v>
       </c>
-      <c r="S18" t="s">
+      <c r="T18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1994,14 +2008,14 @@
       <c r="Q19" t="s">
         <v>197</v>
       </c>
-      <c r="R19" t="s">
+      <c r="S19" t="s">
         <v>154</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2047,11 +2061,11 @@
       <c r="Q20" t="s">
         <v>198</v>
       </c>
-      <c r="R20" t="s">
+      <c r="S20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
feat: add data_size field to dataset with aggregation to folder, institution, and tag
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225553FA-C012-F041-B23D-9037C1595045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA120681-540F-8149-966A-6B132712E9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="210">
   <si>
     <t>id</t>
   </si>
@@ -647,6 +647,9 @@
   </si>
   <si>
     <t>nb_files</t>
+  </si>
+  <si>
+    <t>data_size</t>
   </si>
 </sst>
 </file>
@@ -725,9 +728,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:T21" totalsRowShown="0">
-  <autoFilter ref="A1:T21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:U21" totalsRowShown="0">
+  <autoFilter ref="A1:U21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -746,6 +749,7 @@
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
     <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_files"/>
+    <tableColumn id="20" xr3:uid="{CC390F1F-B31A-914F-918F-4457DB5509B3}" name="data_size"/>
     <tableColumn id="18" xr3:uid="{4730D97E-AE17-A44B-9512-0BF292D5AFB4}" name="tag_ids"/>
     <tableColumn id="19" xr3:uid="{288E2992-818F-AA4B-8F92-E9D2F7E670E8}" name="doc_ids"/>
   </tableColumns>
@@ -1040,7 +1044,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T21"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1060,11 +1064,12 @@
     <col min="16" max="16" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="22.83203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.6640625" customWidth="1"/>
+    <col min="20" max="20" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1120,13 +1125,16 @@
         <v>208</v>
       </c>
       <c r="S1" t="s">
+        <v>209</v>
+      </c>
+      <c r="T1" t="s">
         <v>103</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1169,11 +1177,14 @@
       <c r="Q2" t="s">
         <v>182</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2">
+        <v>134432</v>
+      </c>
+      <c r="T2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1225,11 +1236,14 @@
       <c r="Q3" t="s">
         <v>183</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3">
+        <v>543</v>
+      </c>
+      <c r="T3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:21" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1271,11 +1285,14 @@
       <c r="Q4" t="s">
         <v>184</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="S4">
+        <v>956844335</v>
+      </c>
+      <c r="T4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1311,11 +1328,11 @@
       <c r="Q5" t="s">
         <v>185</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1361,14 +1378,14 @@
       <c r="Q6" t="s">
         <v>186</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>144</v>
       </c>
-      <c r="T6" t="s">
+      <c r="U6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1414,14 +1431,14 @@
       <c r="Q7" t="s">
         <v>187</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>145</v>
       </c>
-      <c r="T7" t="s">
+      <c r="U7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1464,11 +1481,11 @@
       <c r="Q8" t="s">
         <v>188</v>
       </c>
-      <c r="T8" t="s">
+      <c r="U8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1514,11 +1531,11 @@
       <c r="Q9" t="s">
         <v>189</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1561,11 +1578,11 @@
       <c r="Q10" t="s">
         <v>190</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1611,11 +1628,11 @@
       <c r="Q11" t="s">
         <v>191</v>
       </c>
-      <c r="S11" t="s">
+      <c r="T11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1658,14 +1675,14 @@
       <c r="O12" t="s">
         <v>38</v>
       </c>
-      <c r="S12" t="s">
+      <c r="T12" t="s">
         <v>149</v>
       </c>
-      <c r="T12" t="s">
+      <c r="U12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1711,11 +1728,11 @@
       <c r="Q13" t="s">
         <v>192</v>
       </c>
-      <c r="S13" t="s">
+      <c r="T13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1761,11 +1778,11 @@
       <c r="Q14" t="s">
         <v>193</v>
       </c>
-      <c r="T14" t="s">
+      <c r="U14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1814,8 +1831,11 @@
       <c r="R15">
         <v>3</v>
       </c>
+      <c r="S15">
+        <v>958473</v>
+      </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1852,11 +1872,11 @@
       <c r="O16" t="s">
         <v>20</v>
       </c>
-      <c r="S16" t="s">
+      <c r="T16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1902,11 +1922,11 @@
       <c r="Q17" t="s">
         <v>195</v>
       </c>
-      <c r="S17" t="s">
+      <c r="T17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -1955,14 +1975,17 @@
       <c r="R18">
         <v>13</v>
       </c>
-      <c r="S18" t="s">
+      <c r="S18">
+        <v>49274393547</v>
+      </c>
+      <c r="T18" t="s">
         <v>153</v>
       </c>
-      <c r="T18" t="s">
+      <c r="U18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2008,14 +2031,14 @@
       <c r="Q19" t="s">
         <v>197</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>154</v>
       </c>
-      <c r="T19" t="s">
+      <c r="U19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2061,11 +2084,11 @@
       <c r="Q20" t="s">
         <v>198</v>
       </c>
-      <c r="S20" t="s">
+      <c r="T20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
fix: select filter URL encoding and simplify filter persistence to URL-only
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA120681-540F-8149-966A-6B132712E9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC77935-A241-3545-AF32-EFBFE7C0E7B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1976,7 +1976,7 @@
         <v>13</v>
       </c>
       <c r="S18">
-        <v>49274393547</v>
+        <v>49274393543</v>
       </c>
       <c r="T18" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
Add data_size field and fix column filter persistence (#108)
* feat: add data_size field to dataset with aggregation to folder, institution, and tag

* fix: select filter URL encoding and simplify filter persistence to URL-only
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225553FA-C012-F041-B23D-9037C1595045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC77935-A241-3545-AF32-EFBFE7C0E7B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="210">
   <si>
     <t>id</t>
   </si>
@@ -647,6 +647,9 @@
   </si>
   <si>
     <t>nb_files</t>
+  </si>
+  <si>
+    <t>data_size</t>
   </si>
 </sst>
 </file>
@@ -725,9 +728,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:T21" totalsRowShown="0">
-  <autoFilter ref="A1:T21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:U21" totalsRowShown="0">
+  <autoFilter ref="A1:U21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -746,6 +749,7 @@
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
     <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_files"/>
+    <tableColumn id="20" xr3:uid="{CC390F1F-B31A-914F-918F-4457DB5509B3}" name="data_size"/>
     <tableColumn id="18" xr3:uid="{4730D97E-AE17-A44B-9512-0BF292D5AFB4}" name="tag_ids"/>
     <tableColumn id="19" xr3:uid="{288E2992-818F-AA4B-8F92-E9D2F7E670E8}" name="doc_ids"/>
   </tableColumns>
@@ -1040,7 +1044,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T21"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1060,11 +1064,12 @@
     <col min="16" max="16" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="22.83203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.6640625" customWidth="1"/>
+    <col min="20" max="20" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1120,13 +1125,16 @@
         <v>208</v>
       </c>
       <c r="S1" t="s">
+        <v>209</v>
+      </c>
+      <c r="T1" t="s">
         <v>103</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1169,11 +1177,14 @@
       <c r="Q2" t="s">
         <v>182</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2">
+        <v>134432</v>
+      </c>
+      <c r="T2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1225,11 +1236,14 @@
       <c r="Q3" t="s">
         <v>183</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3">
+        <v>543</v>
+      </c>
+      <c r="T3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:21" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1271,11 +1285,14 @@
       <c r="Q4" t="s">
         <v>184</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="S4">
+        <v>956844335</v>
+      </c>
+      <c r="T4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1311,11 +1328,11 @@
       <c r="Q5" t="s">
         <v>185</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1361,14 +1378,14 @@
       <c r="Q6" t="s">
         <v>186</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>144</v>
       </c>
-      <c r="T6" t="s">
+      <c r="U6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1414,14 +1431,14 @@
       <c r="Q7" t="s">
         <v>187</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>145</v>
       </c>
-      <c r="T7" t="s">
+      <c r="U7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1464,11 +1481,11 @@
       <c r="Q8" t="s">
         <v>188</v>
       </c>
-      <c r="T8" t="s">
+      <c r="U8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1514,11 +1531,11 @@
       <c r="Q9" t="s">
         <v>189</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1561,11 +1578,11 @@
       <c r="Q10" t="s">
         <v>190</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1611,11 +1628,11 @@
       <c r="Q11" t="s">
         <v>191</v>
       </c>
-      <c r="S11" t="s">
+      <c r="T11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1658,14 +1675,14 @@
       <c r="O12" t="s">
         <v>38</v>
       </c>
-      <c r="S12" t="s">
+      <c r="T12" t="s">
         <v>149</v>
       </c>
-      <c r="T12" t="s">
+      <c r="U12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1711,11 +1728,11 @@
       <c r="Q13" t="s">
         <v>192</v>
       </c>
-      <c r="S13" t="s">
+      <c r="T13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1761,11 +1778,11 @@
       <c r="Q14" t="s">
         <v>193</v>
       </c>
-      <c r="T14" t="s">
+      <c r="U14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1814,8 +1831,11 @@
       <c r="R15">
         <v>3</v>
       </c>
+      <c r="S15">
+        <v>958473</v>
+      </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1852,11 +1872,11 @@
       <c r="O16" t="s">
         <v>20</v>
       </c>
-      <c r="S16" t="s">
+      <c r="T16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1902,11 +1922,11 @@
       <c r="Q17" t="s">
         <v>195</v>
       </c>
-      <c r="S17" t="s">
+      <c r="T17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -1955,14 +1975,17 @@
       <c r="R18">
         <v>13</v>
       </c>
-      <c r="S18" t="s">
+      <c r="S18">
+        <v>49274393543</v>
+      </c>
+      <c r="T18" t="s">
         <v>153</v>
       </c>
-      <c r="T18" t="s">
+      <c r="U18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2008,14 +2031,14 @@
       <c r="Q19" t="s">
         <v>197</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>154</v>
       </c>
-      <c r="T19" t="s">
+      <c r="U19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2061,11 +2084,11 @@
       <c r="Q20" t="s">
         <v>198</v>
       </c>
-      <c r="S20" t="s">
+      <c r="T20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
add: sample_size field for datasets with frequency extrapolation
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC77935-A241-3545-AF32-EFBFE7C0E7B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197EE767-8F48-4E43-A4C2-DEAEF9F76844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="211">
   <si>
     <t>id</t>
   </si>
@@ -650,6 +650,9 @@
   </si>
   <si>
     <t>data_size</t>
+  </si>
+  <si>
+    <t>sample_size</t>
   </si>
 </sst>
 </file>
@@ -728,9 +731,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:U21" totalsRowShown="0">
-  <autoFilter ref="A1:U21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:V21" totalsRowShown="0">
+  <autoFilter ref="A1:V21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="22">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -739,6 +742,7 @@
     <tableColumn id="6" xr3:uid="{D2392623-916B-E04B-A27E-0D01B8B20172}" name="type"/>
     <tableColumn id="7" xr3:uid="{4D4990DC-E580-924E-A6C8-71E0E49DC440}" name="description"/>
     <tableColumn id="8" xr3:uid="{489A14B1-8FC8-C549-8AE1-29C457B8AA01}" name="nb_row"/>
+    <tableColumn id="22" xr3:uid="{9FF51936-9B9E-A649-B173-D0016776EF21}" name="sample_size"/>
     <tableColumn id="11" xr3:uid="{39B5740A-29A3-4149-AEFD-550E62863529}" name="last_update_date" dataDxfId="3"/>
     <tableColumn id="17" xr3:uid="{40840879-BBAB-7248-8755-9023914314E8}" name="no_more_update" dataDxfId="2"/>
     <tableColumn id="12" xr3:uid="{25BA5CC3-7EA6-8F48-BADD-686749A186ED}" name="updating_each"/>
@@ -1044,7 +1048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1055,21 +1059,22 @@
     <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="52.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="17" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.5" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.6640625" customWidth="1"/>
-    <col min="20" max="20" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5" customWidth="1"/>
+    <col min="10" max="11" width="17" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" customWidth="1"/>
+    <col min="21" max="21" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1094,47 +1099,50 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
+        <v>210</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>14</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>15</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>19</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>8</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>18</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>208</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>209</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>103</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1159,32 +1167,32 @@
       <c r="H2">
         <v>3000</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>123</v>
       </c>
-      <c r="L2" s="1">
+      <c r="M2" s="1">
         <v>2002</v>
       </c>
-      <c r="M2" s="1">
+      <c r="N2" s="1">
         <v>2023</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>26</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>182</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>134432</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1209,41 +1217,41 @@
       <c r="H3">
         <v>10</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>123</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>25</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>20</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>207</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>183</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>543</v>
       </c>
-      <c r="T3" t="s">
+      <c r="U3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1268,31 +1276,31 @@
       <c r="H4">
         <v>43023</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>124</v>
       </c>
-      <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" t="s">
+      <c r="N4" s="1"/>
+      <c r="O4" t="s">
         <v>24</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>21</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>184</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>956844335</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="U4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1317,22 +1325,22 @@
       <c r="H5">
         <v>200</v>
       </c>
-      <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" t="s">
+      <c r="N5" s="1"/>
+      <c r="O5" t="s">
         <v>26</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>38</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>185</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1357,35 +1365,38 @@
       <c r="H6">
         <v>500000</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6">
+        <v>100000</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>123</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="N6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>25</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>21</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>186</v>
       </c>
-      <c r="T6" t="s">
+      <c r="U6" t="s">
         <v>144</v>
       </c>
-      <c r="U6" t="s">
+      <c r="V6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1407,38 +1418,38 @@
       <c r="G7" t="s">
         <v>46</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>124</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="M7" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="N7" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>24</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>20</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" t="s">
         <v>187</v>
       </c>
-      <c r="T7" t="s">
+      <c r="U7" t="s">
         <v>145</v>
       </c>
-      <c r="U7" t="s">
+      <c r="V7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1460,32 +1471,32 @@
       <c r="H8">
         <v>34444</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>123</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="M8" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="N8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>64</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>21</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" t="s">
         <v>188</v>
       </c>
-      <c r="U8" t="s">
+      <c r="V8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1510,32 +1521,32 @@
       <c r="H9">
         <v>32389</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>125</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="M9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="N9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>25</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>38</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" t="s">
         <v>189</v>
       </c>
-      <c r="T9" t="s">
+      <c r="U9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1557,32 +1568,32 @@
       <c r="H10">
         <v>67050</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>124</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="M10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="N10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>65</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>21</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="R10" t="s">
         <v>190</v>
       </c>
-      <c r="T10" t="s">
+      <c r="U10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1607,32 +1618,32 @@
       <c r="H11">
         <v>949563</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>124</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="M11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="N11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O11" t="s">
         <v>26</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>21</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="R11" t="s">
         <v>191</v>
       </c>
-      <c r="T11" t="s">
+      <c r="U11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1657,32 +1668,32 @@
       <c r="H12">
         <v>500000</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>123</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="M12" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M12" s="1" t="s">
+      <c r="N12" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="N12" t="s">
+      <c r="O12" t="s">
         <v>25</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" t="s">
         <v>38</v>
       </c>
-      <c r="T12" t="s">
+      <c r="U12" t="s">
         <v>149</v>
       </c>
-      <c r="U12" t="s">
+      <c r="V12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1707,32 +1718,32 @@
       <c r="H13">
         <v>45699</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>125</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="M13" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="M13" s="1" t="s">
+      <c r="N13" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>24</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>21</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="R13" t="s">
         <v>192</v>
       </c>
-      <c r="T13" t="s">
+      <c r="U13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1757,32 +1768,32 @@
       <c r="H14">
         <v>85005</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>123</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="M14" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M14" s="1" t="s">
+      <c r="N14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>26</v>
       </c>
-      <c r="O14" t="s">
+      <c r="P14" t="s">
         <v>38</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="R14" t="s">
         <v>193</v>
       </c>
-      <c r="U14" t="s">
+      <c r="V14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1807,35 +1818,35 @@
       <c r="H15">
         <v>1144</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>125</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="M15" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="M15" s="1" t="s">
+      <c r="N15" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>25</v>
       </c>
-      <c r="O15" t="s">
+      <c r="P15" t="s">
         <v>21</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="R15" t="s">
         <v>194</v>
       </c>
-      <c r="R15">
+      <c r="S15">
         <v>3</v>
       </c>
-      <c r="S15">
+      <c r="T15">
         <v>958473</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1854,29 +1865,29 @@
       <c r="H16">
         <v>44669</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>124</v>
       </c>
-      <c r="L16" s="1" t="s">
+      <c r="M16" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M16" s="1" t="s">
+      <c r="N16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>24</v>
       </c>
-      <c r="O16" t="s">
+      <c r="P16" t="s">
         <v>20</v>
       </c>
-      <c r="T16" t="s">
+      <c r="U16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1901,32 +1912,32 @@
       <c r="H17">
         <v>75656</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>126</v>
       </c>
-      <c r="L17" s="1" t="s">
+      <c r="M17" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M17" s="1" t="s">
+      <c r="N17" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>64</v>
       </c>
-      <c r="O17" t="s">
+      <c r="P17" t="s">
         <v>21</v>
       </c>
-      <c r="Q17" t="s">
+      <c r="R17" t="s">
         <v>195</v>
       </c>
-      <c r="T17" t="s">
+      <c r="U17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -1951,41 +1962,41 @@
       <c r="H18">
         <v>434</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>124</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="M18" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="M18" s="1" t="s">
+      <c r="N18" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N18" t="s">
+      <c r="O18" t="s">
         <v>25</v>
       </c>
-      <c r="O18" t="s">
+      <c r="P18" t="s">
         <v>38</v>
       </c>
-      <c r="Q18" t="s">
+      <c r="R18" t="s">
         <v>196</v>
       </c>
-      <c r="R18">
+      <c r="S18">
         <v>13</v>
       </c>
-      <c r="S18">
+      <c r="T18">
         <v>49274393543</v>
       </c>
-      <c r="T18" t="s">
+      <c r="U18" t="s">
         <v>153</v>
       </c>
-      <c r="U18" t="s">
+      <c r="V18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2010,35 +2021,35 @@
       <c r="H19">
         <v>47398</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>123</v>
       </c>
-      <c r="L19" s="1" t="s">
+      <c r="M19" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M19" s="1" t="s">
+      <c r="N19" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="N19" t="s">
+      <c r="O19" t="s">
         <v>65</v>
       </c>
-      <c r="O19" t="s">
+      <c r="P19" t="s">
         <v>21</v>
       </c>
-      <c r="Q19" t="s">
+      <c r="R19" t="s">
         <v>197</v>
       </c>
-      <c r="T19" t="s">
+      <c r="U19" t="s">
         <v>154</v>
       </c>
-      <c r="U19" t="s">
+      <c r="V19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2063,32 +2074,32 @@
       <c r="H20">
         <v>97344</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="J20" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>125</v>
       </c>
-      <c r="L20" s="1" t="s">
+      <c r="M20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="M20" s="1" t="s">
+      <c r="N20" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N20" t="s">
+      <c r="O20" t="s">
         <v>26</v>
       </c>
-      <c r="O20" t="s">
+      <c r="P20" t="s">
         <v>21</v>
       </c>
-      <c r="Q20" t="s">
+      <c r="R20" t="s">
         <v>198</v>
       </c>
-      <c r="T20" t="s">
+      <c r="U20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -2113,25 +2124,25 @@
       <c r="H21">
         <v>346</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>125</v>
       </c>
-      <c r="L21" s="1" t="s">
+      <c r="M21" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="M21" s="1" t="s">
+      <c r="N21" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="N21" t="s">
+      <c r="O21" t="s">
         <v>24</v>
       </c>
-      <c r="O21" t="s">
+      <c r="P21" t="s">
         <v>21</v>
       </c>
-      <c r="Q21" t="s">
+      <c r="R21" t="s">
         <v>199</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify equal min/max display and extrapolate frequencies from dataset sample size (#110)
* fix: stats preview showing redundant min/max when values are equal

* add: sample_size field for datasets with frequency extrapolation
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC77935-A241-3545-AF32-EFBFE7C0E7B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197EE767-8F48-4E43-A4C2-DEAEF9F76844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="211">
   <si>
     <t>id</t>
   </si>
@@ -650,6 +650,9 @@
   </si>
   <si>
     <t>data_size</t>
+  </si>
+  <si>
+    <t>sample_size</t>
   </si>
 </sst>
 </file>
@@ -728,9 +731,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:U21" totalsRowShown="0">
-  <autoFilter ref="A1:U21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:V21" totalsRowShown="0">
+  <autoFilter ref="A1:V21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="22">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -739,6 +742,7 @@
     <tableColumn id="6" xr3:uid="{D2392623-916B-E04B-A27E-0D01B8B20172}" name="type"/>
     <tableColumn id="7" xr3:uid="{4D4990DC-E580-924E-A6C8-71E0E49DC440}" name="description"/>
     <tableColumn id="8" xr3:uid="{489A14B1-8FC8-C549-8AE1-29C457B8AA01}" name="nb_row"/>
+    <tableColumn id="22" xr3:uid="{9FF51936-9B9E-A649-B173-D0016776EF21}" name="sample_size"/>
     <tableColumn id="11" xr3:uid="{39B5740A-29A3-4149-AEFD-550E62863529}" name="last_update_date" dataDxfId="3"/>
     <tableColumn id="17" xr3:uid="{40840879-BBAB-7248-8755-9023914314E8}" name="no_more_update" dataDxfId="2"/>
     <tableColumn id="12" xr3:uid="{25BA5CC3-7EA6-8F48-BADD-686749A186ED}" name="updating_each"/>
@@ -1044,7 +1048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1055,21 +1059,22 @@
     <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="52.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="17" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.5" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.6640625" customWidth="1"/>
-    <col min="20" max="20" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5" customWidth="1"/>
+    <col min="10" max="11" width="17" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" customWidth="1"/>
+    <col min="21" max="21" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1094,47 +1099,50 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
+        <v>210</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>14</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>15</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>19</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>8</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>18</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>208</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>209</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>103</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1159,32 +1167,32 @@
       <c r="H2">
         <v>3000</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>123</v>
       </c>
-      <c r="L2" s="1">
+      <c r="M2" s="1">
         <v>2002</v>
       </c>
-      <c r="M2" s="1">
+      <c r="N2" s="1">
         <v>2023</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>26</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>182</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>134432</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1209,41 +1217,41 @@
       <c r="H3">
         <v>10</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>123</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>25</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>20</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>207</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>183</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>543</v>
       </c>
-      <c r="T3" t="s">
+      <c r="U3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1268,31 +1276,31 @@
       <c r="H4">
         <v>43023</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>124</v>
       </c>
-      <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" t="s">
+      <c r="N4" s="1"/>
+      <c r="O4" t="s">
         <v>24</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>21</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>184</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>956844335</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="U4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1317,22 +1325,22 @@
       <c r="H5">
         <v>200</v>
       </c>
-      <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" t="s">
+      <c r="N5" s="1"/>
+      <c r="O5" t="s">
         <v>26</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>38</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>185</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1357,35 +1365,38 @@
       <c r="H6">
         <v>500000</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6">
+        <v>100000</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>123</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="N6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>25</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>21</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>186</v>
       </c>
-      <c r="T6" t="s">
+      <c r="U6" t="s">
         <v>144</v>
       </c>
-      <c r="U6" t="s">
+      <c r="V6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1407,38 +1418,38 @@
       <c r="G7" t="s">
         <v>46</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>124</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="M7" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="N7" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>24</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>20</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" t="s">
         <v>187</v>
       </c>
-      <c r="T7" t="s">
+      <c r="U7" t="s">
         <v>145</v>
       </c>
-      <c r="U7" t="s">
+      <c r="V7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1460,32 +1471,32 @@
       <c r="H8">
         <v>34444</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>123</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="M8" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="N8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>64</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>21</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" t="s">
         <v>188</v>
       </c>
-      <c r="U8" t="s">
+      <c r="V8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1510,32 +1521,32 @@
       <c r="H9">
         <v>32389</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>125</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="M9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="N9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>25</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>38</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" t="s">
         <v>189</v>
       </c>
-      <c r="T9" t="s">
+      <c r="U9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1557,32 +1568,32 @@
       <c r="H10">
         <v>67050</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>124</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="M10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="N10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>65</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>21</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="R10" t="s">
         <v>190</v>
       </c>
-      <c r="T10" t="s">
+      <c r="U10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1607,32 +1618,32 @@
       <c r="H11">
         <v>949563</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>124</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="M11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="N11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O11" t="s">
         <v>26</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>21</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="R11" t="s">
         <v>191</v>
       </c>
-      <c r="T11" t="s">
+      <c r="U11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1657,32 +1668,32 @@
       <c r="H12">
         <v>500000</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>123</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="M12" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M12" s="1" t="s">
+      <c r="N12" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="N12" t="s">
+      <c r="O12" t="s">
         <v>25</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" t="s">
         <v>38</v>
       </c>
-      <c r="T12" t="s">
+      <c r="U12" t="s">
         <v>149</v>
       </c>
-      <c r="U12" t="s">
+      <c r="V12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1707,32 +1718,32 @@
       <c r="H13">
         <v>45699</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>125</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="M13" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="M13" s="1" t="s">
+      <c r="N13" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>24</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>21</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="R13" t="s">
         <v>192</v>
       </c>
-      <c r="T13" t="s">
+      <c r="U13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1757,32 +1768,32 @@
       <c r="H14">
         <v>85005</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>123</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="M14" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M14" s="1" t="s">
+      <c r="N14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>26</v>
       </c>
-      <c r="O14" t="s">
+      <c r="P14" t="s">
         <v>38</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="R14" t="s">
         <v>193</v>
       </c>
-      <c r="U14" t="s">
+      <c r="V14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1807,35 +1818,35 @@
       <c r="H15">
         <v>1144</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>125</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="M15" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="M15" s="1" t="s">
+      <c r="N15" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>25</v>
       </c>
-      <c r="O15" t="s">
+      <c r="P15" t="s">
         <v>21</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="R15" t="s">
         <v>194</v>
       </c>
-      <c r="R15">
+      <c r="S15">
         <v>3</v>
       </c>
-      <c r="S15">
+      <c r="T15">
         <v>958473</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1854,29 +1865,29 @@
       <c r="H16">
         <v>44669</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>124</v>
       </c>
-      <c r="L16" s="1" t="s">
+      <c r="M16" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M16" s="1" t="s">
+      <c r="N16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>24</v>
       </c>
-      <c r="O16" t="s">
+      <c r="P16" t="s">
         <v>20</v>
       </c>
-      <c r="T16" t="s">
+      <c r="U16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1901,32 +1912,32 @@
       <c r="H17">
         <v>75656</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>126</v>
       </c>
-      <c r="L17" s="1" t="s">
+      <c r="M17" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M17" s="1" t="s">
+      <c r="N17" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>64</v>
       </c>
-      <c r="O17" t="s">
+      <c r="P17" t="s">
         <v>21</v>
       </c>
-      <c r="Q17" t="s">
+      <c r="R17" t="s">
         <v>195</v>
       </c>
-      <c r="T17" t="s">
+      <c r="U17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -1951,41 +1962,41 @@
       <c r="H18">
         <v>434</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>124</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="M18" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="M18" s="1" t="s">
+      <c r="N18" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N18" t="s">
+      <c r="O18" t="s">
         <v>25</v>
       </c>
-      <c r="O18" t="s">
+      <c r="P18" t="s">
         <v>38</v>
       </c>
-      <c r="Q18" t="s">
+      <c r="R18" t="s">
         <v>196</v>
       </c>
-      <c r="R18">
+      <c r="S18">
         <v>13</v>
       </c>
-      <c r="S18">
+      <c r="T18">
         <v>49274393543</v>
       </c>
-      <c r="T18" t="s">
+      <c r="U18" t="s">
         <v>153</v>
       </c>
-      <c r="U18" t="s">
+      <c r="V18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2010,35 +2021,35 @@
       <c r="H19">
         <v>47398</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>123</v>
       </c>
-      <c r="L19" s="1" t="s">
+      <c r="M19" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M19" s="1" t="s">
+      <c r="N19" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="N19" t="s">
+      <c r="O19" t="s">
         <v>65</v>
       </c>
-      <c r="O19" t="s">
+      <c r="P19" t="s">
         <v>21</v>
       </c>
-      <c r="Q19" t="s">
+      <c r="R19" t="s">
         <v>197</v>
       </c>
-      <c r="T19" t="s">
+      <c r="U19" t="s">
         <v>154</v>
       </c>
-      <c r="U19" t="s">
+      <c r="V19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2063,32 +2074,32 @@
       <c r="H20">
         <v>97344</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="J20" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>125</v>
       </c>
-      <c r="L20" s="1" t="s">
+      <c r="M20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="M20" s="1" t="s">
+      <c r="N20" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N20" t="s">
+      <c r="O20" t="s">
         <v>26</v>
       </c>
-      <c r="O20" t="s">
+      <c r="P20" t="s">
         <v>21</v>
       </c>
-      <c r="Q20" t="s">
+      <c r="R20" t="s">
         <v>198</v>
       </c>
-      <c r="T20" t="s">
+      <c r="U20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -2113,25 +2124,25 @@
       <c r="H21">
         <v>346</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>125</v>
       </c>
-      <c r="L21" s="1" t="s">
+      <c r="M21" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="M21" s="1" t="s">
+      <c r="N21" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="N21" t="s">
+      <c r="O21" t="s">
         <v>24</v>
       </c>
-      <c r="O21" t="s">
+      <c r="P21" t="s">
         <v>21</v>
       </c>
-      <c r="Q21" t="s">
+      <c r="R21" t="s">
         <v>199</v>
       </c>
     </row>

</xml_diff>

<commit_message>
change: rename nb_files to nb_resources to support tables alongside files
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197EE767-8F48-4E43-A4C2-DEAEF9F76844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2BB162A-C694-8648-AB90-232D1988EABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -646,13 +646,13 @@
     <t>dataset/accident_route.xlsx</t>
   </si>
   <si>
-    <t>nb_files</t>
-  </si>
-  <si>
     <t>data_size</t>
   </si>
   <si>
     <t>sample_size</t>
+  </si>
+  <si>
+    <t>nb_resources</t>
   </si>
 </sst>
 </file>
@@ -752,7 +752,7 @@
     <tableColumn id="16" xr3:uid="{ED3587E2-4956-D94E-81CF-A84E6EFAC119}" name="delivery_format"/>
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
-    <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_files"/>
+    <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_resources"/>
     <tableColumn id="20" xr3:uid="{CC390F1F-B31A-914F-918F-4457DB5509B3}" name="data_size"/>
     <tableColumn id="18" xr3:uid="{4730D97E-AE17-A44B-9512-0BF292D5AFB4}" name="tag_ids"/>
     <tableColumn id="19" xr3:uid="{288E2992-818F-AA4B-8F92-E9D2F7E670E8}" name="doc_ids"/>
@@ -1100,7 +1100,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>9</v>
@@ -1130,10 +1130,10 @@
         <v>18</v>
       </c>
       <c r="S1" t="s">
+        <v>210</v>
+      </c>
+      <c r="T1" t="s">
         <v>208</v>
-      </c>
-      <c r="T1" t="s">
-        <v>209</v>
       </c>
       <c r="U1" t="s">
         <v>103</v>

</xml_diff>

<commit_message>
change: rename nb_files to nb_resources to support tables alongside files (#115)
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197EE767-8F48-4E43-A4C2-DEAEF9F76844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2BB162A-C694-8648-AB90-232D1988EABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -646,13 +646,13 @@
     <t>dataset/accident_route.xlsx</t>
   </si>
   <si>
-    <t>nb_files</t>
-  </si>
-  <si>
     <t>data_size</t>
   </si>
   <si>
     <t>sample_size</t>
+  </si>
+  <si>
+    <t>nb_resources</t>
   </si>
 </sst>
 </file>
@@ -752,7 +752,7 @@
     <tableColumn id="16" xr3:uid="{ED3587E2-4956-D94E-81CF-A84E6EFAC119}" name="delivery_format"/>
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
-    <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_files"/>
+    <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_resources"/>
     <tableColumn id="20" xr3:uid="{CC390F1F-B31A-914F-918F-4457DB5509B3}" name="data_size"/>
     <tableColumn id="18" xr3:uid="{4730D97E-AE17-A44B-9512-0BF292D5AFB4}" name="tag_ids"/>
     <tableColumn id="19" xr3:uid="{288E2992-818F-AA4B-8F92-E9D2F7E670E8}" name="doc_ids"/>
@@ -1100,7 +1100,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>9</v>
@@ -1130,10 +1130,10 @@
         <v>18</v>
       </c>
       <c r="S1" t="s">
+        <v>210</v>
+      </c>
+      <c r="T1" t="s">
         <v>208</v>
-      </c>
-      <c r="T1" t="s">
-        <v>209</v>
       </c>
       <c r="U1" t="s">
         <v>103</v>

</xml_diff>

<commit_message>
Add license fields to folders and datasets
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2BB162A-C694-8648-AB90-232D1988EABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11E940C-9EB7-824F-94DF-97A59ECB4A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="215">
   <si>
     <t>id</t>
   </si>
@@ -653,6 +653,18 @@
   </si>
   <si>
     <t>nb_resources</t>
+  </si>
+  <si>
+    <t>license</t>
+  </si>
+  <si>
+    <t>CC-BY-4.0</t>
+  </si>
+  <si>
+    <t>CC-BY-4.0 - attribution requise</t>
+  </si>
+  <si>
+    <t>https://creativecommons.org/licenses/by/4.0/</t>
   </si>
 </sst>
 </file>
@@ -694,12 +706,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -731,9 +744,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:V21" totalsRowShown="0">
-  <autoFilter ref="A1:V21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:W21" totalsRowShown="0">
+  <autoFilter ref="A1:W21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="23">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -750,6 +763,7 @@
     <tableColumn id="10" xr3:uid="{E9CC3D9F-3681-CE44-9463-02B41A65AEDA}" name="end_date" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{AB83C6F1-9210-B442-AD5A-A3BA93064343}" name="localisation"/>
     <tableColumn id="16" xr3:uid="{ED3587E2-4956-D94E-81CF-A84E6EFAC119}" name="delivery_format"/>
+    <tableColumn id="23" xr3:uid="{C81EA0D5-FCEF-014F-BE6F-51DC189A42C4}" name="license"/>
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
     <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_resources"/>
@@ -1048,7 +1062,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1066,15 +1080,16 @@
     <col min="14" max="14" width="12.5" customWidth="1"/>
     <col min="15" max="15" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.6640625" customWidth="1"/>
-    <col min="21" max="21" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.6640625" customWidth="1"/>
+    <col min="22" max="22" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1124,25 +1139,28 @@
         <v>19</v>
       </c>
       <c r="Q1" t="s">
+        <v>211</v>
+      </c>
+      <c r="R1" t="s">
         <v>8</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>210</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>208</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>103</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1182,17 +1200,20 @@
       <c r="P2" t="s">
         <v>21</v>
       </c>
-      <c r="R2" t="s">
+      <c r="Q2" t="s">
+        <v>212</v>
+      </c>
+      <c r="S2" t="s">
         <v>182</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>134432</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1238,20 +1259,20 @@
       <c r="P3" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>207</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>183</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>543</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1290,17 +1311,17 @@
       <c r="P4" t="s">
         <v>21</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>184</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>956844335</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1333,14 +1354,17 @@
       <c r="P5" t="s">
         <v>38</v>
       </c>
-      <c r="R5" t="s">
+      <c r="Q5" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="S5" t="s">
         <v>185</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1386,17 +1410,17 @@
       <c r="P6" t="s">
         <v>21</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>186</v>
       </c>
-      <c r="U6" t="s">
+      <c r="V6" t="s">
         <v>144</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1439,17 +1463,17 @@
       <c r="P7" t="s">
         <v>20</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>187</v>
       </c>
-      <c r="U7" t="s">
+      <c r="V7" t="s">
         <v>145</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1489,14 +1513,14 @@
       <c r="P8" t="s">
         <v>21</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>188</v>
       </c>
-      <c r="V8" t="s">
+      <c r="W8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1539,14 +1563,14 @@
       <c r="P9" t="s">
         <v>38</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>189</v>
       </c>
-      <c r="U9" t="s">
+      <c r="V9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1586,14 +1610,14 @@
       <c r="P10" t="s">
         <v>21</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>190</v>
       </c>
-      <c r="U10" t="s">
+      <c r="V10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1636,14 +1660,17 @@
       <c r="P11" t="s">
         <v>21</v>
       </c>
-      <c r="R11" t="s">
+      <c r="Q11" t="s">
+        <v>213</v>
+      </c>
+      <c r="S11" t="s">
         <v>191</v>
       </c>
-      <c r="U11" t="s">
+      <c r="V11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1686,14 +1713,14 @@
       <c r="P12" t="s">
         <v>38</v>
       </c>
-      <c r="U12" t="s">
+      <c r="V12" t="s">
         <v>149</v>
       </c>
-      <c r="V12" t="s">
+      <c r="W12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1736,14 +1763,14 @@
       <c r="P13" t="s">
         <v>21</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>192</v>
       </c>
-      <c r="U13" t="s">
+      <c r="V13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1786,14 +1813,14 @@
       <c r="P14" t="s">
         <v>38</v>
       </c>
-      <c r="R14" t="s">
+      <c r="S14" t="s">
         <v>193</v>
       </c>
-      <c r="V14" t="s">
+      <c r="W14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1836,17 +1863,20 @@
       <c r="P15" t="s">
         <v>21</v>
       </c>
-      <c r="R15" t="s">
+      <c r="Q15" t="s">
+        <v>213</v>
+      </c>
+      <c r="S15" t="s">
         <v>194</v>
       </c>
-      <c r="S15">
+      <c r="T15">
         <v>3</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <v>958473</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1883,11 +1913,11 @@
       <c r="P16" t="s">
         <v>20</v>
       </c>
-      <c r="U16" t="s">
+      <c r="V16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1930,14 +1960,14 @@
       <c r="P17" t="s">
         <v>21</v>
       </c>
-      <c r="R17" t="s">
+      <c r="S17" t="s">
         <v>195</v>
       </c>
-      <c r="U17" t="s">
+      <c r="V17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -1980,23 +2010,23 @@
       <c r="P18" t="s">
         <v>38</v>
       </c>
-      <c r="R18" t="s">
+      <c r="S18" t="s">
         <v>196</v>
       </c>
-      <c r="S18">
+      <c r="T18">
         <v>13</v>
       </c>
-      <c r="T18">
+      <c r="U18">
         <v>49274393543</v>
       </c>
-      <c r="U18" t="s">
+      <c r="V18" t="s">
         <v>153</v>
       </c>
-      <c r="V18" t="s">
+      <c r="W18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2039,17 +2069,17 @@
       <c r="P19" t="s">
         <v>21</v>
       </c>
-      <c r="R19" t="s">
+      <c r="S19" t="s">
         <v>197</v>
       </c>
-      <c r="U19" t="s">
+      <c r="V19" t="s">
         <v>154</v>
       </c>
-      <c r="V19" t="s">
+      <c r="W19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2092,14 +2122,14 @@
       <c r="P20" t="s">
         <v>21</v>
       </c>
-      <c r="R20" t="s">
+      <c r="S20" t="s">
         <v>198</v>
       </c>
-      <c r="U20" t="s">
+      <c r="V20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -2142,7 +2172,7 @@
       <c r="P21" t="s">
         <v>21</v>
       </c>
-      <c r="R21" t="s">
+      <c r="S21" t="s">
         <v>199</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add license fields to folders and datasets (#128)
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2BB162A-C694-8648-AB90-232D1988EABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11E940C-9EB7-824F-94DF-97A59ECB4A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="215">
   <si>
     <t>id</t>
   </si>
@@ -653,6 +653,18 @@
   </si>
   <si>
     <t>nb_resources</t>
+  </si>
+  <si>
+    <t>license</t>
+  </si>
+  <si>
+    <t>CC-BY-4.0</t>
+  </si>
+  <si>
+    <t>CC-BY-4.0 - attribution requise</t>
+  </si>
+  <si>
+    <t>https://creativecommons.org/licenses/by/4.0/</t>
   </si>
 </sst>
 </file>
@@ -694,12 +706,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -731,9 +744,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:V21" totalsRowShown="0">
-  <autoFilter ref="A1:V21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:W21" totalsRowShown="0">
+  <autoFilter ref="A1:W21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="23">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -750,6 +763,7 @@
     <tableColumn id="10" xr3:uid="{E9CC3D9F-3681-CE44-9463-02B41A65AEDA}" name="end_date" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{AB83C6F1-9210-B442-AD5A-A3BA93064343}" name="localisation"/>
     <tableColumn id="16" xr3:uid="{ED3587E2-4956-D94E-81CF-A84E6EFAC119}" name="delivery_format"/>
+    <tableColumn id="23" xr3:uid="{C81EA0D5-FCEF-014F-BE6F-51DC189A42C4}" name="license"/>
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
     <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_resources"/>
@@ -1048,7 +1062,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1066,15 +1080,16 @@
     <col min="14" max="14" width="12.5" customWidth="1"/>
     <col min="15" max="15" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.6640625" customWidth="1"/>
-    <col min="21" max="21" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.6640625" customWidth="1"/>
+    <col min="22" max="22" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1124,25 +1139,28 @@
         <v>19</v>
       </c>
       <c r="Q1" t="s">
+        <v>211</v>
+      </c>
+      <c r="R1" t="s">
         <v>8</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>210</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>208</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>103</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1182,17 +1200,20 @@
       <c r="P2" t="s">
         <v>21</v>
       </c>
-      <c r="R2" t="s">
+      <c r="Q2" t="s">
+        <v>212</v>
+      </c>
+      <c r="S2" t="s">
         <v>182</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>134432</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1238,20 +1259,20 @@
       <c r="P3" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>207</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>183</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>543</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1290,17 +1311,17 @@
       <c r="P4" t="s">
         <v>21</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>184</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>956844335</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1333,14 +1354,17 @@
       <c r="P5" t="s">
         <v>38</v>
       </c>
-      <c r="R5" t="s">
+      <c r="Q5" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="S5" t="s">
         <v>185</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1386,17 +1410,17 @@
       <c r="P6" t="s">
         <v>21</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>186</v>
       </c>
-      <c r="U6" t="s">
+      <c r="V6" t="s">
         <v>144</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1439,17 +1463,17 @@
       <c r="P7" t="s">
         <v>20</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>187</v>
       </c>
-      <c r="U7" t="s">
+      <c r="V7" t="s">
         <v>145</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1489,14 +1513,14 @@
       <c r="P8" t="s">
         <v>21</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>188</v>
       </c>
-      <c r="V8" t="s">
+      <c r="W8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1539,14 +1563,14 @@
       <c r="P9" t="s">
         <v>38</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>189</v>
       </c>
-      <c r="U9" t="s">
+      <c r="V9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1586,14 +1610,14 @@
       <c r="P10" t="s">
         <v>21</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>190</v>
       </c>
-      <c r="U10" t="s">
+      <c r="V10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1636,14 +1660,17 @@
       <c r="P11" t="s">
         <v>21</v>
       </c>
-      <c r="R11" t="s">
+      <c r="Q11" t="s">
+        <v>213</v>
+      </c>
+      <c r="S11" t="s">
         <v>191</v>
       </c>
-      <c r="U11" t="s">
+      <c r="V11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1686,14 +1713,14 @@
       <c r="P12" t="s">
         <v>38</v>
       </c>
-      <c r="U12" t="s">
+      <c r="V12" t="s">
         <v>149</v>
       </c>
-      <c r="V12" t="s">
+      <c r="W12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1736,14 +1763,14 @@
       <c r="P13" t="s">
         <v>21</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>192</v>
       </c>
-      <c r="U13" t="s">
+      <c r="V13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1786,14 +1813,14 @@
       <c r="P14" t="s">
         <v>38</v>
       </c>
-      <c r="R14" t="s">
+      <c r="S14" t="s">
         <v>193</v>
       </c>
-      <c r="V14" t="s">
+      <c r="W14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1836,17 +1863,20 @@
       <c r="P15" t="s">
         <v>21</v>
       </c>
-      <c r="R15" t="s">
+      <c r="Q15" t="s">
+        <v>213</v>
+      </c>
+      <c r="S15" t="s">
         <v>194</v>
       </c>
-      <c r="S15">
+      <c r="T15">
         <v>3</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <v>958473</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1883,11 +1913,11 @@
       <c r="P16" t="s">
         <v>20</v>
       </c>
-      <c r="U16" t="s">
+      <c r="V16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1930,14 +1960,14 @@
       <c r="P17" t="s">
         <v>21</v>
       </c>
-      <c r="R17" t="s">
+      <c r="S17" t="s">
         <v>195</v>
       </c>
-      <c r="U17" t="s">
+      <c r="V17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -1980,23 +2010,23 @@
       <c r="P18" t="s">
         <v>38</v>
       </c>
-      <c r="R18" t="s">
+      <c r="S18" t="s">
         <v>196</v>
       </c>
-      <c r="S18">
+      <c r="T18">
         <v>13</v>
       </c>
-      <c r="T18">
+      <c r="U18">
         <v>49274393543</v>
       </c>
-      <c r="U18" t="s">
+      <c r="V18" t="s">
         <v>153</v>
       </c>
-      <c r="V18" t="s">
+      <c r="W18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2039,17 +2069,17 @@
       <c r="P19" t="s">
         <v>21</v>
       </c>
-      <c r="R19" t="s">
+      <c r="S19" t="s">
         <v>197</v>
       </c>
-      <c r="U19" t="s">
+      <c r="V19" t="s">
         <v>154</v>
       </c>
-      <c r="V19" t="s">
+      <c r="W19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2092,14 +2122,14 @@
       <c r="P20" t="s">
         <v>21</v>
       </c>
-      <c r="R20" t="s">
+      <c r="S20" t="s">
         <v>198</v>
       </c>
-      <c r="U20" t="s">
+      <c r="V20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -2142,7 +2172,7 @@
       <c r="P21" t="s">
         <v>21</v>
       </c>
-      <c r="R21" t="s">
+      <c r="S21" t="s">
         <v>199</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update preview data for 0.21.3
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11E940C-9EB7-824F-94DF-97A59ECB4A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BA4AF0-919E-DE47-ACF0-9E458337DBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="216">
   <si>
     <t>id</t>
   </si>
@@ -665,6 +665,9 @@
   </si>
   <si>
     <t>https://creativecommons.org/licenses/by/4.0/</t>
+  </si>
+  <si>
+    <t>has_preview</t>
   </si>
 </sst>
 </file>
@@ -706,13 +709,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -744,9 +746,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:W21" totalsRowShown="0">
-  <autoFilter ref="A1:W21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:X21" totalsRowShown="0">
+  <autoFilter ref="A1:X21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -764,6 +766,7 @@
     <tableColumn id="9" xr3:uid="{AB83C6F1-9210-B442-AD5A-A3BA93064343}" name="localisation"/>
     <tableColumn id="16" xr3:uid="{ED3587E2-4956-D94E-81CF-A84E6EFAC119}" name="delivery_format"/>
     <tableColumn id="23" xr3:uid="{C81EA0D5-FCEF-014F-BE6F-51DC189A42C4}" name="license"/>
+    <tableColumn id="24" xr3:uid="{AADB20C1-2634-1B41-AA0D-EAE55740FAF4}" name="has_preview"/>
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
     <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_resources"/>
@@ -1062,7 +1065,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1081,15 +1084,16 @@
     <col min="15" max="15" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="18" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.6640625" customWidth="1"/>
-    <col min="22" max="22" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.6640625" customWidth="1"/>
+    <col min="23" max="23" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1142,25 +1146,28 @@
         <v>211</v>
       </c>
       <c r="R1" t="s">
+        <v>215</v>
+      </c>
+      <c r="S1" t="s">
         <v>8</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>210</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>208</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>103</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1203,17 +1210,17 @@
       <c r="Q2" t="s">
         <v>212</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>182</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>134432</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1259,20 +1266,23 @@
       <c r="P3" t="s">
         <v>20</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3">
+        <v>1</v>
+      </c>
+      <c r="S3" t="s">
         <v>207</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>183</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>543</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1311,17 +1321,17 @@
       <c r="P4" t="s">
         <v>21</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>184</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>956844335</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1354,17 +1364,17 @@
       <c r="P5" t="s">
         <v>38</v>
       </c>
-      <c r="Q5" s="3" t="s">
+      <c r="Q5" t="s">
         <v>214</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>185</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1410,17 +1420,17 @@
       <c r="P6" t="s">
         <v>21</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>186</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>144</v>
       </c>
-      <c r="W6" t="s">
+      <c r="X6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1463,17 +1473,17 @@
       <c r="P7" t="s">
         <v>20</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>187</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>145</v>
       </c>
-      <c r="W7" t="s">
+      <c r="X7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1493,7 +1503,7 @@
         <v>50</v>
       </c>
       <c r="H8">
-        <v>34444</v>
+        <v>33444</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>51</v>
@@ -1513,14 +1523,14 @@
       <c r="P8" t="s">
         <v>21</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>188</v>
       </c>
-      <c r="W8" t="s">
+      <c r="X8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1563,14 +1573,14 @@
       <c r="P9" t="s">
         <v>38</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>189</v>
       </c>
-      <c r="V9" t="s">
+      <c r="W9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1610,14 +1620,14 @@
       <c r="P10" t="s">
         <v>21</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>190</v>
       </c>
-      <c r="V10" t="s">
+      <c r="W10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1663,14 +1673,14 @@
       <c r="Q11" t="s">
         <v>213</v>
       </c>
-      <c r="S11" t="s">
+      <c r="T11" t="s">
         <v>191</v>
       </c>
-      <c r="V11" t="s">
+      <c r="W11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1713,14 +1723,14 @@
       <c r="P12" t="s">
         <v>38</v>
       </c>
-      <c r="V12" t="s">
+      <c r="W12" t="s">
         <v>149</v>
       </c>
-      <c r="W12" t="s">
+      <c r="X12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1763,14 +1773,14 @@
       <c r="P13" t="s">
         <v>21</v>
       </c>
-      <c r="S13" t="s">
+      <c r="T13" t="s">
         <v>192</v>
       </c>
-      <c r="V13" t="s">
+      <c r="W13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1813,14 +1823,14 @@
       <c r="P14" t="s">
         <v>38</v>
       </c>
-      <c r="S14" t="s">
+      <c r="T14" t="s">
         <v>193</v>
       </c>
-      <c r="W14" t="s">
+      <c r="X14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1866,17 +1876,17 @@
       <c r="Q15" t="s">
         <v>213</v>
       </c>
-      <c r="S15" t="s">
+      <c r="T15" t="s">
         <v>194</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <v>3</v>
       </c>
-      <c r="U15">
+      <c r="V15">
         <v>958473</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1913,11 +1923,11 @@
       <c r="P16" t="s">
         <v>20</v>
       </c>
-      <c r="V16" t="s">
+      <c r="W16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1960,14 +1970,14 @@
       <c r="P17" t="s">
         <v>21</v>
       </c>
-      <c r="S17" t="s">
+      <c r="T17" t="s">
         <v>195</v>
       </c>
-      <c r="V17" t="s">
+      <c r="W17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -2010,23 +2020,23 @@
       <c r="P18" t="s">
         <v>38</v>
       </c>
-      <c r="S18" t="s">
+      <c r="T18" t="s">
         <v>196</v>
       </c>
-      <c r="T18">
+      <c r="U18">
         <v>13</v>
       </c>
-      <c r="U18">
+      <c r="V18">
         <v>49274393543</v>
       </c>
-      <c r="V18" t="s">
+      <c r="W18" t="s">
         <v>153</v>
       </c>
-      <c r="W18" t="s">
+      <c r="X18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2069,17 +2079,17 @@
       <c r="P19" t="s">
         <v>21</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>197</v>
       </c>
-      <c r="V19" t="s">
+      <c r="W19" t="s">
         <v>154</v>
       </c>
-      <c r="W19" t="s">
+      <c r="X19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2122,14 +2132,14 @@
       <c r="P20" t="s">
         <v>21</v>
       </c>
-      <c r="S20" t="s">
+      <c r="T20" t="s">
         <v>198</v>
       </c>
-      <c r="V20" t="s">
+      <c r="W20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -2172,7 +2182,7 @@
       <c r="P21" t="s">
         <v>21</v>
       </c>
-      <c r="S21" t="s">
+      <c r="T21" t="s">
         <v>199</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add explicit preview availability and clickable HTTP paths (#133)
* fix: base dataset and variable preview availability on `has_preview`

Co-authored-by: Copilot <copilot@github.com>

* change: make HTTP(S) `data_path` and `metadata_path` values clickable while keeping other paths copyable

* Update preview data for 0.21.3

---------

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/public/data/db-source/dataset.xlsx
+++ b/public/data/db-source/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11E940C-9EB7-824F-94DF-97A59ECB4A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BA4AF0-919E-DE47-ACF0-9E458337DBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2440" yWindow="600" windowWidth="26360" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="216">
   <si>
     <t>id</t>
   </si>
@@ -665,6 +665,9 @@
   </si>
   <si>
     <t>https://creativecommons.org/licenses/by/4.0/</t>
+  </si>
+  <si>
+    <t>has_preview</t>
   </si>
 </sst>
 </file>
@@ -706,13 +709,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -744,9 +746,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:W21" totalsRowShown="0">
-  <autoFilter ref="A1:W21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
-  <tableColumns count="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}" name="Tableau1" displayName="Tableau1" ref="A1:X21" totalsRowShown="0">
+  <autoFilter ref="A1:X21" xr:uid="{3C584991-6C49-624F-A55E-42748A4CF1EC}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{080E2F00-A22C-534D-B9C4-D8C8D5EB31DA}" name="id"/>
     <tableColumn id="2" xr3:uid="{92BFA972-4C1D-4E43-B990-63C7415BF3D0}" name="folder_id"/>
     <tableColumn id="3" xr3:uid="{39D90AAB-DB99-4842-B7A2-ED8697C478CE}" name="owner_id"/>
@@ -764,6 +766,7 @@
     <tableColumn id="9" xr3:uid="{AB83C6F1-9210-B442-AD5A-A3BA93064343}" name="localisation"/>
     <tableColumn id="16" xr3:uid="{ED3587E2-4956-D94E-81CF-A84E6EFAC119}" name="delivery_format"/>
     <tableColumn id="23" xr3:uid="{C81EA0D5-FCEF-014F-BE6F-51DC189A42C4}" name="license"/>
+    <tableColumn id="24" xr3:uid="{AADB20C1-2634-1B41-AA0D-EAE55740FAF4}" name="has_preview"/>
     <tableColumn id="14" xr3:uid="{7536954D-F305-F647-B54D-43D736B0B7C6}" name="link"/>
     <tableColumn id="15" xr3:uid="{E59E90FD-B1FC-204A-B6BB-8501C30CA936}" name="data_path"/>
     <tableColumn id="21" xr3:uid="{C6B87811-0023-5348-B5FB-9839D119E838}" name="nb_resources"/>
@@ -1062,7 +1065,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -1081,15 +1084,16 @@
     <col min="15" max="15" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="18" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.6640625" customWidth="1"/>
-    <col min="22" max="22" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.6640625" customWidth="1"/>
+    <col min="23" max="23" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1142,25 +1146,28 @@
         <v>211</v>
       </c>
       <c r="R1" t="s">
+        <v>215</v>
+      </c>
+      <c r="S1" t="s">
         <v>8</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>210</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>208</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>103</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1203,17 +1210,17 @@
       <c r="Q2" t="s">
         <v>212</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>182</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>134432</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1259,20 +1266,23 @@
       <c r="P3" t="s">
         <v>20</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3">
+        <v>1</v>
+      </c>
+      <c r="S3" t="s">
         <v>207</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>183</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>543</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1311,17 +1321,17 @@
       <c r="P4" t="s">
         <v>21</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>184</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>956844335</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1354,17 +1364,17 @@
       <c r="P5" t="s">
         <v>38</v>
       </c>
-      <c r="Q5" s="3" t="s">
+      <c r="Q5" t="s">
         <v>214</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>185</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1410,17 +1420,17 @@
       <c r="P6" t="s">
         <v>21</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>186</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>144</v>
       </c>
-      <c r="W6" t="s">
+      <c r="X6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1463,17 +1473,17 @@
       <c r="P7" t="s">
         <v>20</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>187</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>145</v>
       </c>
-      <c r="W7" t="s">
+      <c r="X7" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1493,7 +1503,7 @@
         <v>50</v>
       </c>
       <c r="H8">
-        <v>34444</v>
+        <v>33444</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>51</v>
@@ -1513,14 +1523,14 @@
       <c r="P8" t="s">
         <v>21</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>188</v>
       </c>
-      <c r="W8" t="s">
+      <c r="X8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1563,14 +1573,14 @@
       <c r="P9" t="s">
         <v>38</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>189</v>
       </c>
-      <c r="V9" t="s">
+      <c r="W9" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1610,14 +1620,14 @@
       <c r="P10" t="s">
         <v>21</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>190</v>
       </c>
-      <c r="V10" t="s">
+      <c r="W10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1663,14 +1673,14 @@
       <c r="Q11" t="s">
         <v>213</v>
       </c>
-      <c r="S11" t="s">
+      <c r="T11" t="s">
         <v>191</v>
       </c>
-      <c r="V11" t="s">
+      <c r="W11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1713,14 +1723,14 @@
       <c r="P12" t="s">
         <v>38</v>
       </c>
-      <c r="V12" t="s">
+      <c r="W12" t="s">
         <v>149</v>
       </c>
-      <c r="W12" t="s">
+      <c r="X12" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1763,14 +1773,14 @@
       <c r="P13" t="s">
         <v>21</v>
       </c>
-      <c r="S13" t="s">
+      <c r="T13" t="s">
         <v>192</v>
       </c>
-      <c r="V13" t="s">
+      <c r="W13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1813,14 +1823,14 @@
       <c r="P14" t="s">
         <v>38</v>
       </c>
-      <c r="S14" t="s">
+      <c r="T14" t="s">
         <v>193</v>
       </c>
-      <c r="W14" t="s">
+      <c r="X14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1866,17 +1876,17 @@
       <c r="Q15" t="s">
         <v>213</v>
       </c>
-      <c r="S15" t="s">
+      <c r="T15" t="s">
         <v>194</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <v>3</v>
       </c>
-      <c r="U15">
+      <c r="V15">
         <v>958473</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1913,11 +1923,11 @@
       <c r="P16" t="s">
         <v>20</v>
       </c>
-      <c r="V16" t="s">
+      <c r="W16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1960,14 +1970,14 @@
       <c r="P17" t="s">
         <v>21</v>
       </c>
-      <c r="S17" t="s">
+      <c r="T17" t="s">
         <v>195</v>
       </c>
-      <c r="V17" t="s">
+      <c r="W17" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -2010,23 +2020,23 @@
       <c r="P18" t="s">
         <v>38</v>
       </c>
-      <c r="S18" t="s">
+      <c r="T18" t="s">
         <v>196</v>
       </c>
-      <c r="T18">
+      <c r="U18">
         <v>13</v>
       </c>
-      <c r="U18">
+      <c r="V18">
         <v>49274393543</v>
       </c>
-      <c r="V18" t="s">
+      <c r="W18" t="s">
         <v>153</v>
       </c>
-      <c r="W18" t="s">
+      <c r="X18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2069,17 +2079,17 @@
       <c r="P19" t="s">
         <v>21</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>197</v>
       </c>
-      <c r="V19" t="s">
+      <c r="W19" t="s">
         <v>154</v>
       </c>
-      <c r="W19" t="s">
+      <c r="X19" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -2122,14 +2132,14 @@
       <c r="P20" t="s">
         <v>21</v>
       </c>
-      <c r="S20" t="s">
+      <c r="T20" t="s">
         <v>198</v>
       </c>
-      <c r="V20" t="s">
+      <c r="W20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -2172,7 +2182,7 @@
       <c r="P21" t="s">
         <v>21</v>
       </c>
-      <c r="S21" t="s">
+      <c r="T21" t="s">
         <v>199</v>
       </c>
     </row>

</xml_diff>